<commit_message>
Separated sick and vacation leave into {Month + SL/VL}
</commit_message>
<xml_diff>
--- a/public/templates/LEAVE-TEMPLATE.xlsx
+++ b/public/templates/LEAVE-TEMPLATE.xlsx
@@ -29,12 +29,9 @@
       <text>
         <r>
           <rPr>
-            <b val="true"/>
-            <sz val="9"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">CPMD Timekeeper:
 </t>
@@ -219,11 +216,12 @@
     <numFmt numFmtId="171" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="172" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -239,12 +237,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -336,12 +328,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
+      <sz val="10"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -379,7 +368,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.5999"/>
-        <bgColor rgb="FFE7E6E6"/>
+        <bgColor rgb="FFFF8080"/>
       </patternFill>
     </fill>
     <fill>
@@ -391,7 +380,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -540,302 +529,304 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="73">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="10" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="10" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="10" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="12" fillId="0" borderId="12" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="12" fillId="0" borderId="12" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="13" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="12" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="12" fillId="0" borderId="12" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="13" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="11" fillId="0" borderId="13" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="13" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="6" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="7" borderId="15" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="6" borderId="2" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="7" borderId="15" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="12" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="16" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="16" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -847,8 +838,8 @@
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Normal 2" xfId="20"/>
-    <cellStyle name="Comma 2" xfId="21"/>
+    <cellStyle name="Comma 2" xfId="20"/>
+    <cellStyle name="Normal 2" xfId="21"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -870,7 +861,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFE7E6E6"/>
+      <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -886,10 +877,10 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFC5E0B4"/>
+      <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFF19F9E"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>

</xml_diff>